<commit_message>
commit de atualização, banco de dados
</commit_message>
<xml_diff>
--- a/bin/Debug/out/Siseng/2.151/Importação PPQ - 151ª - 2000.xlsx
+++ b/bin/Debug/out/Siseng/2.151/Importação PPQ - 151ª - 2000.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
-  <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr codeName="EstaPastaDeTrabalho"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucasduarte\source\repos\Orçamento_Industrial\windowsFormOI\bin\Debug\out\Siseng\2.151\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5AC9D72-192A-4C10-81D9-60D70F0BE880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE06EA63-D3AD-4298-9A6B-701A4DCE3D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{ED41ACCA-C901-42B1-9304-FCDE1B2E9B8D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{E7A13C59-1217-46C9-A00A-CC99FACCD677}"/>
   </bookViews>
   <sheets>
     <sheet name="PPQ Entregas" sheetId="1" r:id="rId1"/>
@@ -790,7 +790,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -798,14 +798,14 @@
       <b/>
       <sz val="13"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1141,7 +1141,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1151,42 +1151,42 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="Yu Gothic Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
@@ -1216,29 +1216,12 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="Yu Gothic"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
@@ -1268,23 +1251,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1346,6 +1312,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -1354,13 +1327,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1425,38 +1391,18 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81C3622A-4BAE-4C70-8190-6306E16D8E12}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D87087D-2B3E-4718-8633-A6A9030AD064}">
   <sheetPr codeName="Planilha8"/>
   <dimension ref="A1:I112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>